<commit_message>
Actualizacao de dados do endline beira
</commit_message>
<xml_diff>
--- a/PERFIL_PAM_VERDE_BEIRA_C3_2026.xlsx
+++ b/PERFIL_PAM_VERDE_BEIRA_C3_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://muvamozorg.sharepoint.com/sites/mis.drive/Documentos Partilhados/PROJECTOS/Sistema de Monitoria/Pam_Verde/2026/Baseline_Endline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{5040D066-AE66-F545-AC8C-766D23DB4958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DE1BE19-401E-40C5-AB3F-ACF032A36325}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{5040D066-AE66-F545-AC8C-766D23DB4958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FCD3A10-A5BA-434C-BC5E-35E1627886BE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nomes_das_empreendedoras_Report" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="189">
   <si>
     <t>ID da participante</t>
   </si>
@@ -600,6 +600,9 @@
   </si>
   <si>
     <t xml:space="preserve">Acissa </t>
+  </si>
+  <si>
+    <t>Não Iniciou</t>
   </si>
 </sst>
 </file>
@@ -1073,7 +1076,7 @@
         <v>22</v>
       </c>
       <c r="I3" t="s">
-        <v>17</v>
+        <v>185</v>
       </c>
       <c r="J3" t="s">
         <v>186</v>
@@ -1457,7 +1460,7 @@
         <v>82</v>
       </c>
       <c r="I15" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="J15" t="s">
         <v>187</v>
@@ -1585,7 +1588,7 @@
         <v>13</v>
       </c>
       <c r="I19" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="J19" t="s">
         <v>187</v>
@@ -1937,7 +1940,7 @@
         <v>136</v>
       </c>
       <c r="I30" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="J30" t="s">
         <v>184</v>
@@ -2161,7 +2164,7 @@
         <v>13</v>
       </c>
       <c r="I37" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="J37" t="s">
         <v>184</v>
@@ -2270,6 +2273,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="9a7078cd21229583650f2264465a1c40">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e45437c47114f519c494620e3e4bb67" ns2:_="" ns3:_="">
     <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
@@ -2504,7 +2518,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2513,18 +2527,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91B60EC3-BD84-4E67-9739-9EA7921CE3DB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A712F033-FDF8-4463-9AFB-AD92C5C9AFB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2543,21 +2557,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15098CC0-5FCE-4BE0-8984-72AC220AC74D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91B60EC3-BD84-4E67-9739-9EA7921CE3DB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>